<commit_message>
How it works: start-to-end story, tower film, try it
Opens with one drawing that plays six steps in order (builder plans it in,
line to every flat, kitchen fitted, recharge, pour, top up), then the
drop film through a dusk tower, then the recharge-and-pour demo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Moya_One_Harshita_Handover/Moya_One_Project_Tracker.xlsx
+++ b/Moya_One_Harshita_Handover/Moya_One_Project_Tracker.xlsx
@@ -381,7 +381,7 @@
     <t>Build home page (consumer first, builders teaser)</t>
   </si>
   <si>
-    <t>23 Oct (Harshita): Home built and approved hero in place; Moya1™ added; unconfirmed product lines marked PLACEHOLDER (see Claims). Audit: not a full pass yet. Impeccable detect 0 findings; Taste lint 0 FAIL (1 WARN: Inter flagged as a default face, pinned by DESIGN.md). Taste inspect leaves 2 FAILs as documented exceptions for Vinayak: few-pictures (CLAUDE.md requires SVG/3D and bans stock imagery) and covered-text (sticky 3D stage on phones; floating WhatsApp button).</t>
+    <t>23 Oct (Harshita): Home built and approved hero in place; Moya1™ added; unconfirmed product lines marked PLACEHOLDER (see Claims). Audit: not a full pass yet. Impeccable detect 0 findings; Taste lint 0 FAIL (1 WARN: Inter flagged as a default face, pinned by DESIGN.md). Taste inspect leaves 2 FAILs as documented exceptions for Vinayak: few-pictures (CLAUDE.md requires SVG/3D and bans stock imagery) and covered-text (sticky 3D stage on phones; floating WhatsApp button). | 24 Oct (Harshita): How it works now opens with a start-to-end story: one drawing that plays six steps in order (builder plans it in, line laid to every flat, kitchen fitted, then you recharge, pour, top up), with the steps listed beside it; Pause/Play, tap any step; phones show the picture, the current step and a 1-6 row. Film and Try it follow. All drawings labelled Illustrative; no numbers, no prices, no tech detail; no filter claim kept as PLACEHOLDER. Checked 390px and 1440px (no horizontal scroll), reduced motion (starts paused, finished pictures). Audit: Impeccable detect 0 findings; Taste lint 0 FAIL; inspector FAILs are the documented exceptions (few-pictures: SVG/3D only per CLAUDE.md; drop title sits on a solid ink panel over the film). Fixed: class clash with the home hero, mobile layout, font sizes to tokens.</t>
   </si>
   <si>
     <t>E3</t>
@@ -411,7 +411,7 @@
     <t>Build interactions: recharge demo, app panel, how it works</t>
   </si>
   <si>
-    <t>Keep numbers labelled 'sample' | 23 Oct (Harshita): Home: sample recharge demo, 3D kitchen film, tower climb with floor counter (Illustrative). How it works: scroll-driven 3D journey (tower, then kitchen). | 23 Oct (Harshita): Builders: tower construct mode (floors build in order, line follows, kitchens light).</t>
+    <t>Keep numbers labelled 'sample' | 23 Oct (Harshita): Home: sample recharge demo, 3D kitchen film, tower climb with floor counter (Illustrative). How it works: scroll-driven 3D journey (tower, then kitchen). | 23 Oct (Harshita): Builders: tower construct mode (floors build in order, line follows, kitchens light). | 24 Oct (Harshita): How it works now opens with a start-to-end story: one drawing that plays six steps in order (builder plans it in, line laid to every flat, kitchen fitted, then you recharge, pour, top up), with the steps listed beside it; Pause/Play, tap any step; phones show the picture, the current step and a 1-6 row. Film and Try it follow. All drawings labelled Illustrative; no numbers, no prices, no tech detail; no filter claim kept as PLACEHOLDER. Checked 390px and 1440px (no horizontal scroll), reduced motion (starts paused, finished pictures). Audit: Impeccable detect 0 findings; Taste lint 0 FAIL; inspector FAILs are the documented exceptions (few-pictures: SVG/3D only per CLAUDE.md; drop title sits on a solid ink panel over the film). Fixed: class clash with the home hero, mobile layout, font sizes to tokens.</t>
   </si>
   <si>
     <t>E7</t>

</xml_diff>

<commit_message>
How it works: full-screen scroll-driven start-to-end story
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Moya_One_Harshita_Handover/Moya_One_Project_Tracker.xlsx
+++ b/Moya_One_Harshita_Handover/Moya_One_Project_Tracker.xlsx
@@ -381,7 +381,7 @@
     <t>Build home page (consumer first, builders teaser)</t>
   </si>
   <si>
-    <t>23 Oct (Harshita): Home built and approved hero in place; Moya1™ added; unconfirmed product lines marked PLACEHOLDER (see Claims). Audit: not a full pass yet. Impeccable detect 0 findings; Taste lint 0 FAIL (1 WARN: Inter flagged as a default face, pinned by DESIGN.md). Taste inspect leaves 2 FAILs as documented exceptions for Vinayak: few-pictures (CLAUDE.md requires SVG/3D and bans stock imagery) and covered-text (sticky 3D stage on phones; floating WhatsApp button). | 24 Oct (Harshita): How it works now opens with a start-to-end story: one drawing that plays six steps in order (builder plans it in, line laid to every flat, kitchen fitted, then you recharge, pour, top up), with the steps listed beside it; Pause/Play, tap any step; phones show the picture, the current step and a 1-6 row. Film and Try it follow. All drawings labelled Illustrative; no numbers, no prices, no tech detail; no filter claim kept as PLACEHOLDER. Checked 390px and 1440px (no horizontal scroll), reduced motion (starts paused, finished pictures). Audit: Impeccable detect 0 findings; Taste lint 0 FAIL; inspector FAILs are the documented exceptions (few-pictures: SVG/3D only per CLAUDE.md; drop title sits on a solid ink panel over the film). Fixed: class clash with the home hero, mobile layout, font sizes to tokens.</t>
+    <t>23 Oct (Harshita): Home built and approved hero in place; Moya1™ added; unconfirmed product lines marked PLACEHOLDER (see Claims). Audit: not a full pass yet. Impeccable detect 0 findings; Taste lint 0 FAIL (1 WARN: Inter flagged as a default face, pinned by DESIGN.md). Taste inspect leaves 2 FAILs as documented exceptions for Vinayak: few-pictures (CLAUDE.md requires SVG/3D and bans stock imagery) and covered-text (sticky 3D stage on phones; floating WhatsApp button). | 24 Oct (Harshita): How it works now opens with a start-to-end story: one drawing that plays six steps in order (builder plans it in, line laid to every flat, kitchen fitted, then you recharge, pour, top up), with the steps listed beside it; Pause/Play, tap any step; phones show the picture, the current step and a 1-6 row. Film and Try it follow. All drawings labelled Illustrative; no numbers, no prices, no tech detail; no filter claim kept as PLACEHOLDER. Checked 390px and 1440px (no horizontal scroll), reduced motion (starts paused, finished pictures). Audit: Impeccable detect 0 findings; Taste lint 0 FAIL; inspector FAILs are the documented exceptions (few-pictures: SVG/3D only per CLAUDE.md; drop title sits on a solid ink panel over the film). Fixed: class clash with the home hero, mobile layout, font sizes to tokens. | 24 Oct (Harshita): Per feedback, the start-to-end story is now the full-screen opening: the view is pinned and scrolling moves through the six steps one by one (picture changes, step highlights, progress bar fills); tapping a step scrolls to it. Checked 390px and 1440px, no horizontal scroll, all six steps reached by scroll. Audit: Impeccable detect 0; Taste lint 0 FAIL; inspector 1 FAIL = documented few-pictures exception (SVG/3D only per CLAUDE.md). Fixed: mobile h1 size.</t>
   </si>
   <si>
     <t>E3</t>
@@ -411,7 +411,7 @@
     <t>Build interactions: recharge demo, app panel, how it works</t>
   </si>
   <si>
-    <t>Keep numbers labelled 'sample' | 23 Oct (Harshita): Home: sample recharge demo, 3D kitchen film, tower climb with floor counter (Illustrative). How it works: scroll-driven 3D journey (tower, then kitchen). | 23 Oct (Harshita): Builders: tower construct mode (floors build in order, line follows, kitchens light). | 24 Oct (Harshita): How it works now opens with a start-to-end story: one drawing that plays six steps in order (builder plans it in, line laid to every flat, kitchen fitted, then you recharge, pour, top up), with the steps listed beside it; Pause/Play, tap any step; phones show the picture, the current step and a 1-6 row. Film and Try it follow. All drawings labelled Illustrative; no numbers, no prices, no tech detail; no filter claim kept as PLACEHOLDER. Checked 390px and 1440px (no horizontal scroll), reduced motion (starts paused, finished pictures). Audit: Impeccable detect 0 findings; Taste lint 0 FAIL; inspector FAILs are the documented exceptions (few-pictures: SVG/3D only per CLAUDE.md; drop title sits on a solid ink panel over the film). Fixed: class clash with the home hero, mobile layout, font sizes to tokens.</t>
+    <t>Keep numbers labelled 'sample' | 23 Oct (Harshita): Home: sample recharge demo, 3D kitchen film, tower climb with floor counter (Illustrative). How it works: scroll-driven 3D journey (tower, then kitchen). | 23 Oct (Harshita): Builders: tower construct mode (floors build in order, line follows, kitchens light). | 24 Oct (Harshita): How it works now opens with a start-to-end story: one drawing that plays six steps in order (builder plans it in, line laid to every flat, kitchen fitted, then you recharge, pour, top up), with the steps listed beside it; Pause/Play, tap any step; phones show the picture, the current step and a 1-6 row. Film and Try it follow. All drawings labelled Illustrative; no numbers, no prices, no tech detail; no filter claim kept as PLACEHOLDER. Checked 390px and 1440px (no horizontal scroll), reduced motion (starts paused, finished pictures). Audit: Impeccable detect 0 findings; Taste lint 0 FAIL; inspector FAILs are the documented exceptions (few-pictures: SVG/3D only per CLAUDE.md; drop title sits on a solid ink panel over the film). Fixed: class clash with the home hero, mobile layout, font sizes to tokens. | 24 Oct (Harshita): Per feedback, the start-to-end story is now the full-screen opening: the view is pinned and scrolling moves through the six steps one by one (picture changes, step highlights, progress bar fills); tapping a step scrolls to it. Checked 390px and 1440px, no horizontal scroll, all six steps reached by scroll. Audit: Impeccable detect 0; Taste lint 0 FAIL; inspector 1 FAIL = documented few-pictures exception (SVG/3D only per CLAUDE.md). Fixed: mobile h1 size.</t>
   </si>
   <si>
     <t>E7</t>

</xml_diff>

<commit_message>
How it works: story opens full screen, edge to edge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Moya_One_Harshita_Handover/Moya_One_Project_Tracker.xlsx
+++ b/Moya_One_Harshita_Handover/Moya_One_Project_Tracker.xlsx
@@ -381,7 +381,7 @@
     <t>Build home page (consumer first, builders teaser)</t>
   </si>
   <si>
-    <t>23 Oct (Harshita): Home built and approved hero in place; Moya1™ added; unconfirmed product lines marked PLACEHOLDER (see Claims). Audit: not a full pass yet. Impeccable detect 0 findings; Taste lint 0 FAIL (1 WARN: Inter flagged as a default face, pinned by DESIGN.md). Taste inspect leaves 2 FAILs as documented exceptions for Vinayak: few-pictures (CLAUDE.md requires SVG/3D and bans stock imagery) and covered-text (sticky 3D stage on phones; floating WhatsApp button). | 24 Oct (Harshita): How it works now opens with a start-to-end story: one drawing that plays six steps in order (builder plans it in, line laid to every flat, kitchen fitted, then you recharge, pour, top up), with the steps listed beside it; Pause/Play, tap any step; phones show the picture, the current step and a 1-6 row. Film and Try it follow. All drawings labelled Illustrative; no numbers, no prices, no tech detail; no filter claim kept as PLACEHOLDER. Checked 390px and 1440px (no horizontal scroll), reduced motion (starts paused, finished pictures). Audit: Impeccable detect 0 findings; Taste lint 0 FAIL; inspector FAILs are the documented exceptions (few-pictures: SVG/3D only per CLAUDE.md; drop title sits on a solid ink panel over the film). Fixed: class clash with the home hero, mobile layout, font sizes to tokens. | 24 Oct (Harshita): Per feedback, the start-to-end story is now the full-screen opening: the view is pinned and scrolling moves through the six steps one by one (picture changes, step highlights, progress bar fills); tapping a step scrolls to it. Checked 390px and 1440px, no horizontal scroll, all six steps reached by scroll. Audit: Impeccable detect 0; Taste lint 0 FAIL; inspector 1 FAIL = documented few-pictures exception (SVG/3D only per CLAUDE.md). Fixed: mobile h1 size.</t>
+    <t>23 Oct (Harshita): Home built and approved hero in place; Moya1™ added; unconfirmed product lines marked PLACEHOLDER (see Claims). Audit: not a full pass yet. Impeccable detect 0 findings; Taste lint 0 FAIL (1 WARN: Inter flagged as a default face, pinned by DESIGN.md). Taste inspect leaves 2 FAILs as documented exceptions for Vinayak: few-pictures (CLAUDE.md requires SVG/3D and bans stock imagery) and covered-text (sticky 3D stage on phones; floating WhatsApp button). | 24 Oct (Harshita): How it works now opens with a start-to-end story: one drawing that plays six steps in order (builder plans it in, line laid to every flat, kitchen fitted, then you recharge, pour, top up), with the steps listed beside it; Pause/Play, tap any step; phones show the picture, the current step and a 1-6 row. Film and Try it follow. All drawings labelled Illustrative; no numbers, no prices, no tech detail; no filter claim kept as PLACEHOLDER. Checked 390px and 1440px (no horizontal scroll), reduced motion (starts paused, finished pictures). Audit: Impeccable detect 0 findings; Taste lint 0 FAIL; inspector FAILs are the documented exceptions (few-pictures: SVG/3D only per CLAUDE.md; drop title sits on a solid ink panel over the film). Fixed: class clash with the home hero, mobile layout, font sizes to tokens. | 24 Oct (Harshita): Per feedback, the start-to-end story is now the full-screen opening: the view is pinned and scrolling moves through the six steps one by one (picture changes, step highlights, progress bar fills); tapping a step scrolls to it. Checked 390px and 1440px, no horizontal scroll, all six steps reached by scroll. Audit: Impeccable detect 0; Taste lint 0 FAIL; inspector 1 FAIL = documented few-pictures exception (SVG/3D only per CLAUDE.md). Fixed: mobile h1 size. | 24 Oct (Harshita): Per feedback, the start-to-end story is now a full-bleed, full-screen opening like the film (words on the left as captions, drawing filling the screen, 1-6 row): the view is pinned and scrolling moves through the six steps one by one (picture changes, step highlights, progress bar fills); tapping a step scrolls to it. Checked 390px and 1440px, no horizontal scroll, all six steps reached by scroll. Audit: Impeccable detect 0; Taste lint 0 FAIL; inspector 1 FAIL = documented few-pictures exception (SVG/3D only per CLAUDE.md). Fixed: mobile h1 size.</t>
   </si>
   <si>
     <t>E3</t>
@@ -411,7 +411,7 @@
     <t>Build interactions: recharge demo, app panel, how it works</t>
   </si>
   <si>
-    <t>Keep numbers labelled 'sample' | 23 Oct (Harshita): Home: sample recharge demo, 3D kitchen film, tower climb with floor counter (Illustrative). How it works: scroll-driven 3D journey (tower, then kitchen). | 23 Oct (Harshita): Builders: tower construct mode (floors build in order, line follows, kitchens light). | 24 Oct (Harshita): How it works now opens with a start-to-end story: one drawing that plays six steps in order (builder plans it in, line laid to every flat, kitchen fitted, then you recharge, pour, top up), with the steps listed beside it; Pause/Play, tap any step; phones show the picture, the current step and a 1-6 row. Film and Try it follow. All drawings labelled Illustrative; no numbers, no prices, no tech detail; no filter claim kept as PLACEHOLDER. Checked 390px and 1440px (no horizontal scroll), reduced motion (starts paused, finished pictures). Audit: Impeccable detect 0 findings; Taste lint 0 FAIL; inspector FAILs are the documented exceptions (few-pictures: SVG/3D only per CLAUDE.md; drop title sits on a solid ink panel over the film). Fixed: class clash with the home hero, mobile layout, font sizes to tokens. | 24 Oct (Harshita): Per feedback, the start-to-end story is now the full-screen opening: the view is pinned and scrolling moves through the six steps one by one (picture changes, step highlights, progress bar fills); tapping a step scrolls to it. Checked 390px and 1440px, no horizontal scroll, all six steps reached by scroll. Audit: Impeccable detect 0; Taste lint 0 FAIL; inspector 1 FAIL = documented few-pictures exception (SVG/3D only per CLAUDE.md). Fixed: mobile h1 size.</t>
+    <t>Keep numbers labelled 'sample' | 23 Oct (Harshita): Home: sample recharge demo, 3D kitchen film, tower climb with floor counter (Illustrative). How it works: scroll-driven 3D journey (tower, then kitchen). | 23 Oct (Harshita): Builders: tower construct mode (floors build in order, line follows, kitchens light). | 24 Oct (Harshita): How it works now opens with a start-to-end story: one drawing that plays six steps in order (builder plans it in, line laid to every flat, kitchen fitted, then you recharge, pour, top up), with the steps listed beside it; Pause/Play, tap any step; phones show the picture, the current step and a 1-6 row. Film and Try it follow. All drawings labelled Illustrative; no numbers, no prices, no tech detail; no filter claim kept as PLACEHOLDER. Checked 390px and 1440px (no horizontal scroll), reduced motion (starts paused, finished pictures). Audit: Impeccable detect 0 findings; Taste lint 0 FAIL; inspector FAILs are the documented exceptions (few-pictures: SVG/3D only per CLAUDE.md; drop title sits on a solid ink panel over the film). Fixed: class clash with the home hero, mobile layout, font sizes to tokens. | 24 Oct (Harshita): Per feedback, the start-to-end story is now the full-screen opening: the view is pinned and scrolling moves through the six steps one by one (picture changes, step highlights, progress bar fills); tapping a step scrolls to it. Checked 390px and 1440px, no horizontal scroll, all six steps reached by scroll. Audit: Impeccable detect 0; Taste lint 0 FAIL; inspector 1 FAIL = documented few-pictures exception (SVG/3D only per CLAUDE.md). Fixed: mobile h1 size. | 24 Oct (Harshita): Per feedback, the start-to-end story is now a full-bleed, full-screen opening like the film (words on the left as captions, drawing filling the screen, 1-6 row): the view is pinned and scrolling moves through the six steps one by one (picture changes, step highlights, progress bar fills); tapping a step scrolls to it. Checked 390px and 1440px, no horizontal scroll, all six steps reached by scroll. Audit: Impeccable detect 0; Taste lint 0 FAIL; inspector 1 FAIL = documented few-pictures exception (SVG/3D only per CLAUDE.md). Fixed: mobile h1 size.</t>
   </si>
   <si>
     <t>E7</t>

</xml_diff>